<commit_message>
Indonesia-2026 Added: - .flake8 - .pre-commit-config.yaml - README.md - pyproject.toml - sitecustomize.py - tex-fmt.toml Modified: - 2025-Bill.xlsx
</commit_message>
<xml_diff>
--- a/Huracan/2025-Bill.xlsx
+++ b/Huracan/2025-Bill.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10824"/>
   <workbookPr showInkAnnotation="0" checkCompatibility="1" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Akseldkw/Desktop/Aksel/Diving/Huracan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3982822E-484C-F946-A2AA-18E98C3E9E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD524E07-6C4E-A049-9F79-00635C1A9ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,12 +238,14 @@
       <sz val="36"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -251,6 +253,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -287,6 +290,7 @@
       <sz val="18"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -294,6 +298,7 @@
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -438,7 +443,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -532,13 +537,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="57">
     <cellStyle name="Followed Hyperlink" xfId="46" builtinId="9" hidden="1"/>
@@ -1146,28 +1150,28 @@
       <c r="D16" s="4"/>
       <c r="E16" s="30"/>
       <c r="F16" s="4"/>
-      <c r="K16" s="42"/>
-      <c r="L16" s="42" t="s">
+      <c r="K16" s="41"/>
+      <c r="L16" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="M16" s="42" t="s">
+      <c r="M16" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="N16" s="42" t="s">
+      <c r="N16" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="O16" s="42" t="s">
+      <c r="O16" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="P16" s="42" t="s">
+      <c r="P16" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="Q16" s="42" t="s">
+      <c r="Q16" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="42"/>
-      <c r="T16" s="42" t="s">
+      <c r="R16" s="41"/>
+      <c r="S16" s="41"/>
+      <c r="T16" s="41" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1197,38 +1201,38 @@
         <f>F17*12.5%</f>
         <v>1562.5</v>
       </c>
-      <c r="K17" s="42" t="s">
+      <c r="K17" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="L17" s="42">
+      <c r="L17" s="41">
         <f>2500 + 75 + 2*10 + 12</f>
         <v>2607</v>
       </c>
-      <c r="M17" s="42">
+      <c r="M17" s="41">
         <f>2500 + 75 + 2*10 + 6*50</f>
         <v>2895</v>
       </c>
-      <c r="N17" s="42">
+      <c r="N17" s="41">
         <f>1900 + 10 + 75</f>
         <v>1985</v>
       </c>
-      <c r="O17" s="42">
+      <c r="O17" s="41">
         <f>2500 + 2*10 + 6*50</f>
         <v>2820</v>
       </c>
-      <c r="P17" s="42">
+      <c r="P17" s="41">
         <f>2500 + 75 + 2*10 + 6*50 + 210</f>
         <v>3105</v>
       </c>
-      <c r="Q17" s="42">
+      <c r="Q17" s="41">
         <f>2500 + 75 + 2*10 + 6*50 + 66</f>
         <v>2961</v>
       </c>
-      <c r="R17" s="42"/>
-      <c r="S17" s="42" t="s">
+      <c r="R17" s="41"/>
+      <c r="S17" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="T17" s="42">
+      <c r="T17" s="41">
         <f>SUM(L17:Q17)</f>
         <v>16373</v>
       </c>
@@ -1257,16 +1261,16 @@
         <f>F18*0.125</f>
         <v>0</v>
       </c>
-      <c r="K18" s="42"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="42"/>
-      <c r="N18" s="42"/>
-      <c r="O18" s="42"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="42"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="42"/>
-      <c r="T18" s="42">
+      <c r="K18" s="41"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="41"/>
+      <c r="N18" s="41"/>
+      <c r="O18" s="41"/>
+      <c r="P18" s="41"/>
+      <c r="Q18" s="41"/>
+      <c r="R18" s="41"/>
+      <c r="S18" s="41"/>
+      <c r="T18" s="41">
         <f t="shared" ref="T18:T26" si="1">SUM(L18:Q18)</f>
         <v>0</v>
       </c>
@@ -1295,21 +1299,21 @@
         <f>H19*L19</f>
         <v>0</v>
       </c>
-      <c r="K19" s="42">
+      <c r="K19" s="41">
         <f>H19*0.09</f>
         <v>0</v>
       </c>
-      <c r="L19" s="42">
+      <c r="L19" s="41">
         <v>1.0900000000000001</v>
       </c>
-      <c r="M19" s="42"/>
-      <c r="N19" s="42"/>
-      <c r="O19" s="42"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="42"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="42"/>
-      <c r="T19" s="42">
+      <c r="M19" s="41"/>
+      <c r="N19" s="41"/>
+      <c r="O19" s="41"/>
+      <c r="P19" s="41"/>
+      <c r="Q19" s="41"/>
+      <c r="R19" s="41"/>
+      <c r="S19" s="41"/>
+      <c r="T19" s="41">
         <f t="shared" si="1"/>
         <v>1.0900000000000001</v>
       </c>
@@ -1338,21 +1342,21 @@
         <f>H20*L20</f>
         <v>0</v>
       </c>
-      <c r="K20" s="42">
+      <c r="K20" s="41">
         <f>H20*0.125</f>
         <v>0</v>
       </c>
-      <c r="L20" s="42">
+      <c r="L20" s="41">
         <v>1.125</v>
       </c>
-      <c r="M20" s="42"/>
-      <c r="N20" s="42"/>
-      <c r="O20" s="42"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="42"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="42"/>
-      <c r="T20" s="42">
+      <c r="M20" s="41"/>
+      <c r="N20" s="41"/>
+      <c r="O20" s="41"/>
+      <c r="P20" s="41"/>
+      <c r="Q20" s="41"/>
+      <c r="R20" s="41"/>
+      <c r="S20" s="41"/>
+      <c r="T20" s="41">
         <f t="shared" si="1"/>
         <v>1.125</v>
       </c>
@@ -1381,21 +1385,21 @@
         <f>H21*L21</f>
         <v>0</v>
       </c>
-      <c r="K21" s="42">
+      <c r="K21" s="41">
         <f>$H21*0.125</f>
         <v>0</v>
       </c>
-      <c r="L21" s="42">
+      <c r="L21" s="41">
         <v>1.125</v>
       </c>
-      <c r="M21" s="42"/>
-      <c r="N21" s="42"/>
-      <c r="O21" s="42"/>
-      <c r="P21" s="42"/>
-      <c r="Q21" s="42"/>
-      <c r="R21" s="42"/>
-      <c r="S21" s="42"/>
-      <c r="T21" s="42">
+      <c r="M21" s="41"/>
+      <c r="N21" s="41"/>
+      <c r="O21" s="41"/>
+      <c r="P21" s="41"/>
+      <c r="Q21" s="41"/>
+      <c r="R21" s="41"/>
+      <c r="S21" s="41"/>
+      <c r="T21" s="41">
         <f t="shared" si="1"/>
         <v>1.125</v>
       </c>
@@ -1427,16 +1431,16 @@
         <f>F22*0.125</f>
         <v>0</v>
       </c>
-      <c r="K22" s="42"/>
-      <c r="L22" s="42"/>
-      <c r="M22" s="42"/>
-      <c r="N22" s="42"/>
-      <c r="O22" s="42"/>
-      <c r="P22" s="42"/>
-      <c r="Q22" s="42"/>
-      <c r="R22" s="42"/>
-      <c r="S22" s="42"/>
-      <c r="T22" s="42">
+      <c r="K22" s="41"/>
+      <c r="L22" s="41"/>
+      <c r="M22" s="41"/>
+      <c r="N22" s="41"/>
+      <c r="O22" s="41"/>
+      <c r="P22" s="41"/>
+      <c r="Q22" s="41"/>
+      <c r="R22" s="41"/>
+      <c r="S22" s="41"/>
+      <c r="T22" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1463,16 +1467,16 @@
         <f>F23*12.5%</f>
         <v>0</v>
       </c>
-      <c r="K23" s="42"/>
-      <c r="L23" s="42"/>
-      <c r="M23" s="42"/>
-      <c r="N23" s="42"/>
-      <c r="O23" s="42"/>
-      <c r="P23" s="42"/>
-      <c r="Q23" s="42"/>
-      <c r="R23" s="42"/>
-      <c r="S23" s="42"/>
-      <c r="T23" s="42">
+      <c r="K23" s="41"/>
+      <c r="L23" s="41"/>
+      <c r="M23" s="41"/>
+      <c r="N23" s="41"/>
+      <c r="O23" s="41"/>
+      <c r="P23" s="41"/>
+      <c r="Q23" s="41"/>
+      <c r="R23" s="41"/>
+      <c r="S23" s="41"/>
+      <c r="T23" s="41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1503,38 +1507,38 @@
         <f>SUM(F24*12.5%)</f>
         <v>237.5</v>
       </c>
-      <c r="K24" s="42" t="s">
+      <c r="K24" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="L24" s="42">
+      <c r="L24" s="41">
         <f>L17 *12.5%</f>
         <v>325.875</v>
       </c>
-      <c r="M24" s="42">
+      <c r="M24" s="41">
         <f t="shared" ref="M24:Q24" si="2">M17 *12.5%</f>
         <v>361.875</v>
       </c>
-      <c r="N24" s="42">
+      <c r="N24" s="41">
         <f t="shared" si="2"/>
         <v>248.125</v>
       </c>
-      <c r="O24" s="42">
+      <c r="O24" s="41">
         <f t="shared" si="2"/>
         <v>352.5</v>
       </c>
-      <c r="P24" s="42">
+      <c r="P24" s="41">
         <f t="shared" si="2"/>
         <v>388.125</v>
       </c>
-      <c r="Q24" s="42">
+      <c r="Q24" s="41">
         <f t="shared" si="2"/>
         <v>370.125</v>
       </c>
-      <c r="R24" s="42"/>
-      <c r="S24" s="42" t="s">
+      <c r="R24" s="41"/>
+      <c r="S24" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="T24" s="42">
+      <c r="T24" s="41">
         <f t="shared" si="1"/>
         <v>2046.625</v>
       </c>
@@ -1569,38 +1573,38 @@
         <f>SUM(F25*12.5%)</f>
         <v>150</v>
       </c>
-      <c r="K25" s="42" t="s">
+      <c r="K25" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="L25" s="42">
+      <c r="L25" s="41">
         <f>L17*20%</f>
         <v>521.4</v>
       </c>
-      <c r="M25" s="42">
+      <c r="M25" s="41">
         <f t="shared" ref="M25:Q25" si="3">M17*20%</f>
         <v>579</v>
       </c>
-      <c r="N25" s="42">
+      <c r="N25" s="41">
         <f t="shared" si="3"/>
         <v>397</v>
       </c>
-      <c r="O25" s="42">
+      <c r="O25" s="41">
         <f t="shared" si="3"/>
         <v>564</v>
       </c>
-      <c r="P25" s="42">
+      <c r="P25" s="41">
         <f t="shared" si="3"/>
         <v>621</v>
       </c>
-      <c r="Q25" s="42">
+      <c r="Q25" s="41">
         <f t="shared" si="3"/>
         <v>592.20000000000005</v>
       </c>
-      <c r="R25" s="42"/>
-      <c r="S25" s="42" t="s">
+      <c r="R25" s="41"/>
+      <c r="S25" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="T25" s="42">
+      <c r="T25" s="41">
         <f t="shared" si="1"/>
         <v>3274.6000000000004</v>
       </c>
@@ -1630,38 +1634,38 @@
         <f>SUM(H26*12.5%)</f>
         <v>37.5</v>
       </c>
-      <c r="K26" s="42" t="s">
+      <c r="K26" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="L26" s="42">
+      <c r="L26" s="41">
         <f>L17+L24+L25</f>
         <v>3454.2750000000001</v>
       </c>
-      <c r="M26" s="42">
+      <c r="M26" s="41">
         <f t="shared" ref="M26:Q26" si="4">M17+M24+M25</f>
         <v>3835.875</v>
       </c>
-      <c r="N26" s="42">
+      <c r="N26" s="41">
         <f t="shared" si="4"/>
         <v>2630.125</v>
       </c>
-      <c r="O26" s="42">
+      <c r="O26" s="41">
         <f t="shared" si="4"/>
         <v>3736.5</v>
       </c>
-      <c r="P26" s="42">
+      <c r="P26" s="41">
         <f t="shared" si="4"/>
         <v>4114.125</v>
       </c>
-      <c r="Q26" s="42">
+      <c r="Q26" s="41">
         <f t="shared" si="4"/>
         <v>3923.3249999999998</v>
       </c>
-      <c r="R26" s="42"/>
-      <c r="S26" s="42" t="s">
+      <c r="R26" s="41"/>
+      <c r="S26" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="T26" s="42">
+      <c r="T26" s="41">
         <f t="shared" si="1"/>
         <v>21694.225000000002</v>
       </c>
@@ -1692,38 +1696,38 @@
         <f>F27*0</f>
         <v>0</v>
       </c>
-      <c r="K27" s="42" t="s">
+      <c r="K27" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="L27" s="42">
+      <c r="L27" s="41">
         <f>L26-3900/6</f>
         <v>2804.2750000000001</v>
       </c>
-      <c r="M27" s="42">
+      <c r="M27" s="41">
         <f t="shared" ref="M27:Q27" si="5">M26-3900/6</f>
         <v>3185.875</v>
       </c>
-      <c r="N27" s="42">
+      <c r="N27" s="41">
         <f t="shared" si="5"/>
         <v>1980.125</v>
       </c>
-      <c r="O27" s="42">
+      <c r="O27" s="41">
         <f t="shared" si="5"/>
         <v>3086.5</v>
       </c>
-      <c r="P27" s="42">
+      <c r="P27" s="41">
         <f t="shared" si="5"/>
         <v>3464.125</v>
       </c>
-      <c r="Q27" s="42">
+      <c r="Q27" s="41">
         <f t="shared" si="5"/>
         <v>3273.3249999999998</v>
       </c>
-      <c r="R27" s="42"/>
-      <c r="S27" s="42" t="s">
+      <c r="R27" s="41"/>
+      <c r="S27" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="T27" s="43">
+      <c r="T27" s="42">
         <f>T26-F35</f>
         <v>17794.225000000002</v>
       </c>
@@ -1816,11 +1820,10 @@
       <c r="D31" s="4"/>
       <c r="E31" s="30"/>
       <c r="F31" s="8"/>
-      <c r="G31" s="44">
+      <c r="G31" s="43">
         <f>SUM(F17:F28)</f>
         <v>16010</v>
       </c>
-      <c r="H31" s="45"/>
     </row>
     <row r="32" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A32" s="4"/>
@@ -1903,12 +1906,12 @@
     </row>
     <row r="40" spans="1:8" ht="54" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B40" s="23"/>
-      <c r="C40" s="41" t="s">
+      <c r="C40" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="41"/>
-      <c r="E40" s="41"/>
-      <c r="F40" s="41"/>
+      <c r="D40" s="44"/>
+      <c r="E40" s="44"/>
+      <c r="F40" s="44"/>
     </row>
     <row r="41" spans="1:8" ht="15" hidden="1" x14ac:dyDescent="0.2"/>
   </sheetData>

</xml_diff>